<commit_message>
Update roles and soundingPurpose dictionaries
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10719"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/Documents/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FABE5D-137B-0A4F-B799-B86CCD48F052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D499BC-A13A-CF43-95D1-F488862FB7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9900" yWindow="3640" windowWidth="34440" windowHeight="20320" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="294">
   <si>
     <t>Description</t>
   </si>
@@ -900,6 +900,24 @@
   </si>
   <si>
     <t>//diggs:samplingFeature//diggs:rolePerformed</t>
+  </si>
+  <si>
+    <t>The on-site engineer associated with this feature or activity</t>
+  </si>
+  <si>
+    <t>field_engineer</t>
+  </si>
+  <si>
+    <t>Field Engineer</t>
+  </si>
+  <si>
+    <t>geologist</t>
+  </si>
+  <si>
+    <t>Geologist</t>
+  </si>
+  <si>
+    <t>The on-site geologist associated with this feature or activity</t>
   </si>
 </sst>
 </file>
@@ -1030,17 +1048,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1058,62 +1076,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="21">
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="0"/>
-      </font>
-    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1202,6 +1164,62 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="0"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium7"/>
   <extLst>
@@ -1216,53 +1234,53 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:E3" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="12"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H16" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
-  <autoFilter ref="A1:H16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H18" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H18" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="7">
       <calculatedColumnFormula>IF(ISNA(VLOOKUP(B2,AssociatedElements!B$2:B2836,1,FALSE)),"Not used","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="11">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="6">
       <calculatedColumnFormula>SUBSTITUTE(SUBSTITUTE(LOWER(Definitions[[#This Row],[Name]])," ","_"),"/","_")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="AssociatedElements" displayName="AssociatedElements" ref="A1:D22" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:D22" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="AssociatedElements" displayName="AssociatedElements" ref="A1:D24" totalsRowShown="0" headerRowDxfId="20">
+  <autoFilter ref="A1:D24" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D22">
     <sortCondition ref="B1:B22"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Start" dataDxfId="3">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Start" dataDxfId="19">
       <calculatedColumnFormula>IF(ISNA(VLOOKUP(B2,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="ID" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="SourceElement" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="ConditionalElement" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="ID" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="SourceElement" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="ConditionalElement" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1608,7 +1626,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.1640625" style="2" customWidth="1"/>
@@ -1949,7 +1967,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="15" t="str">
+      <c r="A16" s="2" t="str">
         <f>IF(ISNA(VLOOKUP(B16,AssociatedElements!B$2:B2850,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
@@ -1959,13 +1977,55 @@
       <c r="C16" s="11" t="s">
         <v>280</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="11" t="s">
         <v>281</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>4</v>
       </c>
       <c r="G16" s="10" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="13" t="str">
+        <f>IF(ISNA(VLOOKUP(B17,AssociatedElements!B$2:B2851,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" s="13" t="str">
+        <f>IF(ISNA(VLOOKUP(B18,AssociatedElements!B$2:B2852,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" s="10" t="s">
         <v>232</v>
       </c>
     </row>
@@ -1981,7 +2041,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.1640625" customWidth="1"/>
@@ -2044,11 +2104,11 @@
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="str">
+      <c r="A5" t="str">
         <f>IF(ISNA(VLOOKUP(B5,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="11" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -2057,14 +2117,14 @@
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="12" t="str">
+      <c r="A6" t="str">
         <f>IF(ISNA(VLOOKUP(B6,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="11" t="s">
         <v>269</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="12" t="s">
         <v>286</v>
       </c>
       <c r="D6" s="2"/>
@@ -2083,11 +2143,11 @@
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="str">
+      <c r="A8" t="str">
         <f>IF(ISNA(VLOOKUP(B8,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="11" t="s">
         <v>253</v>
       </c>
       <c r="C8" s="4" t="s">
@@ -2109,11 +2169,11 @@
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="str">
+      <c r="A10" t="str">
         <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="11" t="s">
         <v>260</v>
       </c>
       <c r="C10" s="4" t="s">
@@ -2148,14 +2208,14 @@
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="str">
+      <c r="A13" t="str">
         <f>IF(ISNA(VLOOKUP(B13,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="11" t="s">
         <v>255</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="12" t="s">
         <v>268</v>
       </c>
       <c r="D13" s="2"/>
@@ -2174,11 +2234,11 @@
       <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="12" t="str">
+      <c r="A15" t="str">
         <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="11" t="s">
         <v>252</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -2200,11 +2260,11 @@
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="str">
+      <c r="A17" t="str">
         <f>IF(ISNA(VLOOKUP(B17,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="11" t="s">
         <v>251</v>
       </c>
       <c r="C17" s="4" t="s">
@@ -2276,6 +2336,32 @@
         <v>261</v>
       </c>
       <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="15" t="str">
+        <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" s="15" t="str">
+        <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1840,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D24" s="2"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C2">

</xml_diff>

<commit_message>
R11 - contractType and governingSpecificationSource dictionaries; widen owner/client
Two new codelists, bound to the new diggs:Contract fields:
contractType.xml (design_build, design_bid_build - Design row 6, contract
delivery method, closed as a side effect of R11) and
governingSpecificationSource.xml (owner_or_agency_provisions,
contractor_specifications, none). Both survey-sourced (RI-DIGGS Technical
Report Table 3-1), authority=DIGGS.

roles.xml: widened owner/client from //diggs:project//diggs:rolePerformed
to the general //diggs:rolePerformed, matching main_contractor/
specialty_contractor's already-working pattern in the same file - both
were unusably scoped to Project-only, which blocked stating who chose the
governing spec on RIProgramBasis/role or Contract/role, neither of which
nests inside Project.
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>//diggs:project//diggs:rolePerformed</t>
+          <t>//diggs:rolePerformed</t>
         </is>
       </c>
       <c r="D4" s="13" t="n"/>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>//diggs:project//diggs:rolePerformed</t>
+          <t>//diggs:rolePerformed</t>
         </is>
       </c>
       <c r="D18" s="13" t="n"/>

</xml_diff>